<commit_message>
Update loco downloads 2026-04-05 15:56:55
</commit_message>
<xml_diff>
--- a/downloads/loco_database.xlsx
+++ b/downloads/loco_database.xlsx
@@ -4056,7 +4056,11 @@
         </is>
       </c>
       <c r="B215" t="inlineStr"/>
-      <c r="C215" t="inlineStr"/>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>PN Toll Freight</t>
+        </is>
+      </c>
       <c r="D215" t="inlineStr">
         <is>
           <t>2026-04-05 15:26:42</t>
@@ -7399,7 +7403,11 @@
         </is>
       </c>
       <c r="B424" t="inlineStr"/>
-      <c r="C424" t="inlineStr"/>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Aurizon Empty Grain</t>
+        </is>
+      </c>
       <c r="D424" t="inlineStr">
         <is>
           <t>2026-04-05 01:09:16</t>
@@ -7577,7 +7585,11 @@
         </is>
       </c>
       <c r="B435" t="inlineStr"/>
-      <c r="C435" t="inlineStr"/>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Hunter Line Service</t>
+        </is>
+      </c>
       <c r="D435" t="inlineStr">
         <is>
           <t>2026-04-03 15:09:22</t>
@@ -22586,7 +22598,11 @@
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PN Toll Freight</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>2026-04-05 15:26:42</t>
@@ -24916,7 +24932,11 @@
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Aurizon Empty Grain</t>
+        </is>
+      </c>
       <c r="D135" t="inlineStr">
         <is>
           <t>2026-04-05 01:09:16</t>
@@ -33245,7 +33265,11 @@
         </is>
       </c>
       <c r="B617" t="inlineStr"/>
-      <c r="C617" t="inlineStr"/>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Hunter Line Service</t>
+        </is>
+      </c>
       <c r="D617" t="inlineStr">
         <is>
           <t>2026-04-03 15:09:22</t>

</xml_diff>

<commit_message>
Update frontend loco download files
</commit_message>
<xml_diff>
--- a/downloads/loco_database.xlsx
+++ b/downloads/loco_database.xlsx
@@ -5998,7 +5998,7 @@
       <c r="B315" t="inlineStr"/>
       <c r="C315" t="inlineStr">
         <is>
-          <t>PN Local Shunter</t>
+          <t>PN Grain Shuttle</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
@@ -11755,7 +11755,7 @@
       <c r="B652" t="inlineStr"/>
       <c r="C652" t="inlineStr">
         <is>
-          <t>Hunter Line Service</t>
+          <t>Hunter Railcar Transfer</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
@@ -18819,7 +18819,7 @@
       <c r="B1048" t="inlineStr"/>
       <c r="C1048" t="inlineStr">
         <is>
-          <t>Upfield Line</t>
+          <t>Craigieburn Line</t>
         </is>
       </c>
       <c r="D1048" t="inlineStr">
@@ -19107,7 +19107,7 @@
       <c r="B1064" t="inlineStr"/>
       <c r="C1064" t="inlineStr">
         <is>
-          <t>Craigieburn Line</t>
+          <t>Upfield Line</t>
         </is>
       </c>
       <c r="D1064" t="inlineStr">
@@ -37916,7 +37916,7 @@
       <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
-          <t>PN Local Shunter</t>
+          <t>PN Grain Shuttle</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -51238,7 +51238,7 @@
       <c r="B841" t="inlineStr"/>
       <c r="C841" t="inlineStr">
         <is>
-          <t>Hunter Line Service</t>
+          <t>Hunter Railcar Transfer</t>
         </is>
       </c>
       <c r="D841" t="inlineStr">
@@ -51670,7 +51670,7 @@
       <c r="B865" t="inlineStr"/>
       <c r="C865" t="inlineStr">
         <is>
-          <t>Upfield Line</t>
+          <t>Craigieburn Line</t>
         </is>
       </c>
       <c r="D865" t="inlineStr">
@@ -63211,7 +63211,7 @@
       <c r="B1512" t="inlineStr"/>
       <c r="C1512" t="inlineStr">
         <is>
-          <t>Craigieburn Line</t>
+          <t>Upfield Line</t>
         </is>
       </c>
       <c r="D1512" t="inlineStr">

</xml_diff>